<commit_message>
add example xlsx on main page
</commit_message>
<xml_diff>
--- a/example/example_log.xlsx
+++ b/example/example_log.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="46">
   <si>
     <t>Date</t>
   </si>
@@ -147,10 +147,10 @@
     <t>Activated charcoal</t>
   </si>
   <si>
-    <t>Diet supplement: Fiber, just one day</t>
+    <t>stop</t>
   </si>
   <si>
-    <t>stop</t>
+    <t>Diet supplement: Fiber, just one day</t>
   </si>
 </sst>
 </file>
@@ -12923,8 +12923,14 @@
     </row>
     <row r="13">
       <c r="A13" s="12"/>
+      <c r="B13" s="32" t="s">
+        <v>43</v>
+      </c>
+      <c r="C13" s="32" t="s">
+        <v>44</v>
+      </c>
       <c r="D13" s="32" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="14">
@@ -12959,10 +12965,10 @@
         <v>40</v>
       </c>
       <c r="C21" s="32" t="s">
+        <v>44</v>
+      </c>
+      <c r="D21" s="32" t="s">
         <v>45</v>
-      </c>
-      <c r="D21" s="32" t="s">
-        <v>44</v>
       </c>
     </row>
     <row r="22">

</xml_diff>